<commit_message>
updated BOM for Haushofer
</commit_message>
<xml_diff>
--- a/Bestuecker_UZ_Digital_Optical_18Tx_14Tx4Rx_v3/BOM_Digital_Optical_18Tx_14Tx4Rx_3vxx_3v01.xlsx
+++ b/Bestuecker_UZ_Digital_Optical_18Tx_14Tx4Rx_v3/BOM_Digital_Optical_18Tx_14Tx4Rx_3vxx_3v01.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ga92wum\git\UltraZohm\PCB\ultrazohm_digital_optical_16tx_3rx_2vxx\Project Outputs for Digital_Optical_18Tx_14Tx4Rx_3vxx\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ga92wum\git\UltraZohm\PCB\ultrazohm_digital_optical_16tx_3rx_2vxx\Bestuecker_UZ_Digital_Optical_18Tx_14Tx4Rx_v3\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="H8" s="47">
         <f ca="1">NOW()</f>
-        <v>44067.501458333332</v>
+        <v>44067.601465509259</v>
       </c>
       <c r="I8" s="28"/>
       <c r="J8" s="28"/>

</xml_diff>